<commit_message>
docs: restructure course outline with categories
</commit_message>
<xml_diff>
--- a/RL_NPU_Course_Outline.xlsx
+++ b/RL_NPU_Course_Outline.xlsx
@@ -33,11 +33,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -55,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -69,21 +69,47 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,204 +475,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>模块</t>
+          <t>课程分类</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>知识点</t>
+          <t>课程</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>时长</t>
+          <t>章节</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>实操</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="80" customHeight="1">
+          <t>链接</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1. RL 训推分离架构</t>
+          <t>快速入门</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>• 三进程模型：Inference(vLLM) / Trainer(torchrun) / Orchestrator(CPU)
-• 权重同步：filesystem vs NCCL，NPU 上必须用 filesystem
-• Launcher 进程管理与僵尸清理</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>画架构图
-启动一次训练观察三进程
-模拟崩溃清理僵尸</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="80" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2. Rollout 生成与采样</t>
-        </is>
-      </c>
+          <t>环境搭建</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>CANN 驱动与 torch_npu 安装 / npu-smi 排卡与 ASCEND_RT_VISIBLE_DEVICES / pip 华为云镜像配置</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="5" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>• batch_size vs group_size：组内共享 prompt 做 group scoring
-• Data Parallel 推理：dp=6 并行生成 1024 条 rollout
-• vLLM Ascend 要点：gpu_memory_utilization=0.8，V1 引擎 hang 排查</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>调 batch/group 看 rollout 量变化
-curl vLLM API 验证推理可用性</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>3. Reward 与 Advantage</t>
-        </is>
-      </c>
+          <t>模型下载与验证</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>HuggingFace 模型下载与本地缓存 / SFT 权重格式(safetensors)校验 / 基模 vs SFT 权重的 Reward 差异</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="6" t="n"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>• Wordle 环境：verifiers → TextArena，格式/部分/胜利三层奖励
-• GRPO 简化 advantage：reward - group_mean
-• Filters：gibberish/repetition/zero_advantage 过滤无效 rollout</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>打印单局 Wordle 完整 reward
-手动计算 advantage 对比框架输出</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
+          <t>RL 训练启动</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>rl_npu.toml 最小配置解析 / 一行命令启动训推分离 / 观察三进程日志(orch/trainer/infer)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4. RL 训练循环</t>
+          <t>进阶开发</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>• Policy Gradient 直觉：好动作提概率，坏动作降
-• PPO 三件套：importance ratio / clipping / KL 约束
-• 关键指标：Loss≠Reward，RL 看 reward 不看 loss</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>追踪一次前向的 loss 计算链路
-同时盯 Loss/Reward/Entropy/GradNorm 四指标</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>5. RL 超参调优</t>
-        </is>
-      </c>
+          <t>RL 训推分离架构</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>三进程协作：Inference / Trainer / Orchestrator / Filesystem 权重同步 vs NCCL / Launcher 进程管理与僵尸清理</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="5" t="n"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>• batch_size：小 batch→梯度噪声大(GradNorm 飙 4亿)，大 batch→稳定但慢
-• lr：1e-6 权重爆炸，1e-7 稳定 29 步，RL 对 lr 比 SFT 敏感
-• dtype：bf16→NaN(log_softmax 词表 152064 溢出)，fp32→稳定但 OOM
-• seq_len：Wordle 6轮×150token≈900，1024 刚好</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>A/B 测试 batch=8/16/32
-对比 lr=1e-6 vs 1e-7
-bf16 vs fp32 各跑 10 步</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>6. RL 特有问题排查</t>
-        </is>
-      </c>
+          <t>Rollout 生成与采样</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>batch_size vs group_size / Data Parallel 推理 / max_completion_tokens 与 Truncation / vLLM Ascend 适配(gpu_mem=0.8, V1 hang)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="5" t="n"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>• NaN logprob → vLLM 400 错误，排查链路：orch→infer→trainer
-• Rollout inflight 挂起 → V1 async hang，curl 诊断→换卡或 V0
-• ACL 硬件异常 → 507015(nonzero)可 workaround，507035(vector core)硬件层</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>复现 NaN 并修复
-触发 inflight hang 并诊断
-收集不同 ACL error code</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>7. RL 训练日志解读</t>
-        </is>
-      </c>
+          <t>Reward 与 Advantage</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Wordle 三层奖励(格式/部分/胜利) / GRPO advantage：reward-group_mean / Filters 过滤无效 rollout</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="5" t="n"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>• Orchestrator：Reward 曲线、Turns 上升=学会多轮、Error% 监控
-• Trainer：Entropy 波动=不稳定、MismatchKL&gt;0.01=策略偏移、PeakMem
-• W&amp;B offline：本地记录，对比多次实验曲线</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>分析 29 步日志画趋势图
-标注 GradNorm 异常点
-算各指标间相关性</t>
-        </is>
-      </c>
+          <t>RL 训练循环</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Policy Gradient 直觉 / PPO: importance ratio + clipping + KL 约束 / Loss 不降≠训练失败，Reward 才是目标</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>RL 超参调优</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>batch_size 对梯度稳定性的影响(GradNorm 4亿→1) / lr 选择(1e-6 爆炸 vs 1e-7 稳定) / bf16 NaN vs fp32 OOM 取舍 / seq_len 与 Truncation</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>RL 训练日志解读</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Orchestrator：Reward/Turns/Error%/Truncation / Trainer：Loss/Entropy/MismatchKL/GradNorm/PeakMem / W&amp;B offline 多实验对比</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CUDA→NPU 代码迁移</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>设备抽象层 _device.py 设计 / 50+ 处硬编码替换 / CUDA 包条件 import(ring_flash_attn, dion) / HCCL 替代 NCCL</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>高阶应用</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>acl 硬件异常排查</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>aclnnNonzeroV2(507015) 与 boolean mask workaround / MTE vector core(507035) 硬件级异常 / NPU→CPU copy 同步故障</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>大规模 RL 训练</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>多卡分布式：DP/TP/CP/EP 取舍 / batch_size 扩展(1024 → 8 的 128x 差距) / 训推比调优与吞吐优化 / 生产级稳定性与断点续训</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>开发中</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A5:A11"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: simplify course outline - single category, RL pipeline only
</commit_message>
<xml_diff>
--- a/RL_NPU_Course_Outline.xlsx
+++ b/RL_NPU_Course_Outline.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -94,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,11 +97,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -475,12 +467,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
@@ -512,7 +504,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>快速入门</t>
@@ -520,246 +512,138 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>环境搭建</t>
+          <t>RL 训推分离架构</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>CANN 驱动与 torch_npu 安装 / npu-smi 排卡与 ASCEND_RT_VISIBLE_DEVICES / pip 华为云镜像配置</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr">
+          <t>三进程协作(Inference/Trainer/Orchestrator) / 权重同步与数据流转</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="5" t="n"/>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="4" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>模型下载与验证</t>
+          <t>Rollout 生成与采样</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>HuggingFace 模型下载与本地缓存 / SFT 权重格式(safetensors)校验 / 基模 vs SFT 权重的 Reward 差异</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
+          <t>batch_size 与 group_size / Data Parallel 推理 / vLLM Ascend 适配</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="6" t="n"/>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="4" t="n"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>RL 训练启动</t>
+          <t>Reward 与 Advantage</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>rl_npu.toml 最小配置解析 / 一行命令启动训推分离 / 观察三进程日志(orch/trainer/infer)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
+          <t>Wordle 环境评分 / GRPO advantage 计算 / rollout 过滤器</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>进阶开发</t>
-        </is>
-      </c>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="n"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>RL 训推分离架构</t>
+          <t>RL 训练循环</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>三进程协作：Inference / Trainer / Orchestrator / Filesystem 权重同步 vs NCCL / Launcher 进程管理与僵尸清理</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
+          <t>Policy Gradient / PPO(importance ratio + clipping + KL) / 关键指标解读</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="5" t="n"/>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="n"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Rollout 生成与采样</t>
+          <t>RL 超参调优</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>batch_size vs group_size / Data Parallel 推理 / max_completion_tokens 与 Truncation / vLLM Ascend 适配(gpu_mem=0.8, V1 hang)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
+          <t>batch_size 与梯度稳定性 / lr 选择 / bf16 vs fp32 / seq_len 权衡</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="n"/>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="n"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Reward 与 Advantage</t>
+          <t>RL 问题排查</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Wordle 三层奖励(格式/部分/胜利) / GRPO advantage：reward-group_mean / Filters 过滤无效 rollout</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
+          <t>NaN logprob / rollout inflight 挂起 / Grad Norm 爆炸 / acl 硬件异常</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>RL 训练循环</t>
+          <t>RL 日志解读</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Policy Gradient 直觉 / PPO: importance ratio + clipping + KL 约束 / Loss 不降≠训练失败，Reward 才是目标</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
+          <t>Orchestrator(Reward/Turns/Error) / Trainer(Loss/Entropy/GradNorm/MFU) / W&amp;B</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>RL 超参调优</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>batch_size 对梯度稳定性的影响(GradNorm 4亿→1) / lr 选择(1e-6 爆炸 vs 1e-7 稳定) / bf16 NaN vs fp32 OOM 取舍 / seq_len 与 Truncation</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>RL 训练日志解读</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Orchestrator：Reward/Turns/Error%/Truncation / Trainer：Loss/Entropy/MismatchKL/GradNorm/PeakMem / W&amp;B offline 多实验对比</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>CUDA→NPU 代码迁移</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>设备抽象层 _device.py 设计 / 50+ 处硬编码替换 / CUDA 包条件 import(ring_flash_attn, dion) / HCCL 替代 NCCL</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>高阶应用</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>acl 硬件异常排查</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>aclnnNonzeroV2(507015) 与 boolean mask workaround / MTE vector core(507035) 硬件级异常 / NPU→CPU copy 同步故障</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>大规模 RL 训练</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>多卡分布式：DP/TP/CP/EP 取舍 / batch_size 扩展(1024 → 8 的 128x 差距) / 训推比调优与吞吐优化 / 生产级稳定性与断点续训</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A5:A11"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: trim course outline to 4 essentials
</commit_message>
<xml_diff>
--- a/RL_NPU_Course_Outline.xlsx
+++ b/RL_NPU_Course_Outline.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -512,12 +512,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>RL 训推分离架构</t>
+          <t>RL 训练启动</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>三进程协作(Inference/Trainer/Orchestrator) / 权重同步与数据流转</t>
+          <t>训推分离架构 / rl_npu.toml 最小配置 / 一行命令启动 / 三进程日志定位</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -531,12 +531,12 @@
       <c r="A3" s="4" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Rollout 生成与采样</t>
+          <t>Rollout 与 Reward</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>batch_size 与 group_size / Data Parallel 推理 / vLLM Ascend 适配</t>
+          <t>batch_size/group_size 设置 / Wordle 环境评分 / vLLM Ascend 推理适配</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -550,12 +550,12 @@
       <c r="A4" s="4" t="n"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Reward 与 Advantage</t>
+          <t>RL 训练与调参</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Wordle 环境评分 / GRPO advantage 计算 / rollout 过滤器</t>
+          <t>Policy Gradient + PPO 训练循环 / lr/batch/dtype/seq_len 调优 / 关键指标速查</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -566,76 +566,19 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="4" t="n"/>
+      <c r="A5" s="5" t="n"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>RL 训练循环</t>
+          <t>常见问题排查</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Policy Gradient / PPO(importance ratio + clipping + KL) / 关键指标解读</t>
+          <t>NaN logprob / rollout 挂起 / Grad Norm 爆炸 / acl 硬件异常 / 僵尸进程清理</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>RL 超参调优</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>batch_size 与梯度稳定性 / lr 选择 / bf16 vs fp32 / seq_len 权衡</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>RL 问题排查</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>NaN logprob / rollout inflight 挂起 / Grad Norm 爆炸 / acl 硬件异常</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>开发中</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>RL 日志解读</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Orchestrator(Reward/Turns/Error) / Trainer(Loss/Entropy/GradNorm/MFU) / W&amp;B</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>开发中</t>
         </is>
@@ -643,7 +586,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A2:A5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>